<commit_message>
UPDATE: atualização de código, remoção de bugs e arquivos não utilizados.
</commit_message>
<xml_diff>
--- a/app/backend/src/modules/Memorial/memorial_prenchido.xlsx
+++ b/app/backend/src/modules/Memorial/memorial_prenchido.xlsx
@@ -1578,7 +1578,7 @@
     <row r="8" ht="14.15" customHeight="1" s="134">
       <c r="B8" s="151" t="inlineStr">
         <is>
-          <t>JA1</t>
+          <t>Alvenaria a demolir</t>
         </is>
       </c>
       <c r="C8" s="140" t="n"/>
@@ -1629,7 +1629,7 @@
     <row r="9" ht="14.15" customHeight="1" s="134">
       <c r="B9" s="154" t="inlineStr">
         <is>
-          <t>JR1</t>
+          <t>Janelas a remover</t>
         </is>
       </c>
       <c r="C9" s="140" t="n"/>
@@ -1676,7 +1676,7 @@
     <row r="10" ht="14.15" customHeight="1" s="134">
       <c r="B10" s="154" t="inlineStr">
         <is>
-          <t>JA2</t>
+          <t>Alvenaria Estrutural a construir</t>
         </is>
       </c>
       <c r="C10" s="140" t="n"/>
@@ -1723,7 +1723,7 @@
     <row r="11" ht="14.15" customHeight="1" s="134">
       <c r="B11" s="154" t="inlineStr">
         <is>
-          <t>JF1</t>
+          <t>Portas a instalar</t>
         </is>
       </c>
       <c r="C11" s="140" t="n"/>
@@ -1770,7 +1770,7 @@
     <row r="12" ht="14.15" customHeight="1" s="134">
       <c r="B12" s="154" t="inlineStr">
         <is>
-          <t>JA4</t>
+          <t>Divisórias em Drywall a construir (espessura = 10cm)</t>
         </is>
       </c>
       <c r="C12" s="140" t="n"/>
@@ -1817,7 +1817,7 @@
     <row r="13" ht="14.15" customHeight="1" s="134">
       <c r="B13" s="154" t="inlineStr">
         <is>
-          <t>JA3</t>
+          <t>Janelas a instalar</t>
         </is>
       </c>
       <c r="C13" s="140" t="n"/>
@@ -1862,7 +1862,7 @@
     <row r="14" ht="14.15" customHeight="1" s="134">
       <c r="B14" s="154" t="inlineStr">
         <is>
-          <t>PM1</t>
+          <t>Radier (espessura = 20cm)</t>
         </is>
       </c>
       <c r="C14" s="140" t="n"/>
@@ -1907,7 +1907,7 @@
     <row r="15" ht="14.15" customHeight="1" s="134">
       <c r="B15" s="154" t="inlineStr">
         <is>
-          <t>PM2</t>
+          <t>TOM. ALTA</t>
         </is>
       </c>
       <c r="C15" s="140" t="n"/>
@@ -1952,7 +1952,7 @@
     <row r="16" ht="14.15" customHeight="1" s="134">
       <c r="B16" s="154" t="inlineStr">
         <is>
-          <t>PV1</t>
+          <t>TOM. MÉDIA</t>
         </is>
       </c>
       <c r="C16" s="140" t="n"/>
@@ -1997,7 +1997,7 @@
     <row r="17" ht="14.15" customHeight="1" s="134">
       <c r="B17" s="154" t="inlineStr">
         <is>
-          <t>PD1</t>
+          <t>TOM.  BAIXA</t>
         </is>
       </c>
       <c r="C17" s="140" t="n"/>
@@ -2042,7 +2042,7 @@
     <row r="18" ht="14.15" customHeight="1" s="134">
       <c r="B18" s="154" t="inlineStr">
         <is>
-          <t>PA1</t>
+          <t>EMERGÊNCIA</t>
         </is>
       </c>
       <c r="C18" s="140" t="n"/>
@@ -2087,7 +2087,7 @@
     <row r="19" ht="14.15" customHeight="1" s="134">
       <c r="B19" s="154" t="inlineStr">
         <is>
-          <t>PM3</t>
+          <t>INTERRUPTOR SIMPLES</t>
         </is>
       </c>
       <c r="C19" s="140" t="n"/>
@@ -2132,7 +2132,7 @@
     <row r="20" ht="14.15" customHeight="1" s="134">
       <c r="B20" s="154" t="inlineStr">
         <is>
-          <t>BAIXA</t>
+          <t>QDG/QD</t>
         </is>
       </c>
       <c r="C20" s="140" t="n"/>
@@ -2177,7 +2177,7 @@
     <row r="21" ht="14.15" customHeight="1" s="134">
       <c r="B21" s="154" t="inlineStr">
         <is>
-          <t>MÉDIA</t>
+          <t>LUMINÁRIA TIPO CALHA 2X36W</t>
         </is>
       </c>
       <c r="C21" s="140" t="n"/>
@@ -2222,7 +2222,7 @@
     <row r="22" ht="14.15" customHeight="1" s="134">
       <c r="B22" s="154" t="inlineStr">
         <is>
-          <t>ALTA</t>
+          <t>CONDUÍTE</t>
         </is>
       </c>
       <c r="C22" s="140" t="n"/>
@@ -2267,7 +2267,7 @@
     <row r="23" ht="14.15" customHeight="1" s="134">
       <c r="B23" s="154" t="inlineStr">
         <is>
-          <t>\pi-0.3,l0.45,t0.45;INTERRUPTOR</t>
+          <t>ELETROCALHA</t>
         </is>
       </c>
       <c r="C23" s="140" t="n"/>
@@ -2312,7 +2312,7 @@
     <row r="24" ht="14.15" customHeight="1" s="134">
       <c r="B24" s="154" t="inlineStr">
         <is>
-          <t>\pxqc;ALOJAMENTO</t>
+          <t>CIRCUITO</t>
         </is>
       </c>
       <c r="C24" s="140" t="n"/>
@@ -2357,7 +2357,7 @@
     <row r="25" ht="14.15" customHeight="1" s="134">
       <c r="B25" s="154" t="inlineStr">
         <is>
-          <t>\pxqc;BANHEIRO 1</t>
+          <t>INST./LOCAL</t>
         </is>
       </c>
       <c r="C25" s="140" t="n"/>
@@ -2402,7 +2402,7 @@
     <row r="26" ht="14.15" customHeight="1" s="134">
       <c r="B26" s="154" t="inlineStr">
         <is>
-          <t>\pxqc;COPA</t>
+          <t>TOMADA/AUDITÓRIO</t>
         </is>
       </c>
       <c r="C26" s="140" t="n"/>
@@ -2447,7 +2447,7 @@
     <row r="27" ht="14.15" customHeight="1" s="134">
       <c r="B27" s="154" t="inlineStr">
         <is>
-          <t>\pxqc;PASSADIÇO</t>
+          <t>ILUM. TOM. AR/ALJ4</t>
         </is>
       </c>
       <c r="C27" s="140" t="n"/>

</xml_diff>